<commit_message>
Fix S25-120/S35-120 specs from Robot_spec.xlsx, add CAD files, update versions to 26.04.17.01
</commit_message>
<xml_diff>
--- a/InoRobotSelect/temp_spec.xlsx
+++ b/InoRobotSelect/temp_spec.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b96646d0fc390357/Desktop/made_C^N/InoRobotAssistant/InoRobotSelect/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="323" documentId="8_{522FA3AE-843B-45F5-9EBE-713FE4E8C55E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E12D8BA1-58AD-432E-AC83-292119DE4DDD}"/>
+  <xr:revisionPtr revIDLastSave="325" documentId="8_{522FA3AE-843B-45F5-9EBE-713FE4E8C55E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C1AC83C-ED8D-492F-A7A3-DBE17A4A05C7}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{166C1812-565C-44F3-A85A-A23A1F110762}"/>
+    <workbookView xWindow="28680" yWindow="-3270" windowWidth="18240" windowHeight="28320" activeTab="3" xr2:uid="{166C1812-565C-44F3-A85A-A23A1F110762}"/>
   </bookViews>
   <sheets>
     <sheet name="6-Axis" sheetId="3" r:id="rId1"/>
@@ -367,9 +367,6 @@
     <t>IR-S25-120Z36C-INT</t>
   </si>
   <si>
-    <t>IR-S35-80Z35C-INT</t>
-  </si>
-  <si>
     <t>IR-S35-100Z35C-INT</t>
   </si>
   <si>
@@ -1140,6 +1137,10 @@
   </si>
   <si>
     <t>IP20</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>IR-S35-80Z35C-INT</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -2324,88 +2325,88 @@
         <v>0</v>
       </c>
       <c r="B1" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="C1" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="D1" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="E1" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="F1" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="G1" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="H1" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="I1" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="H1" s="20" t="s">
-        <v>295</v>
-      </c>
-      <c r="I1" s="20" t="s">
+      <c r="J1" s="20" t="s">
         <v>166</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="K1" s="20" t="s">
         <v>167</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="L1" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="M1" s="20" t="s">
         <v>169</v>
-      </c>
-      <c r="M1" s="20" t="s">
-        <v>170</v>
       </c>
       <c r="N1" s="9"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="21" t="s">
+        <v>170</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>171</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="C2" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="D2" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="E2" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="F2" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="G2" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="H2" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="I2" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="J2" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="K2" s="17" t="s">
         <v>180</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="L2" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="L2" s="17" t="s">
+      <c r="M2" s="17" t="s">
         <v>182</v>
-      </c>
-      <c r="M2" s="17" t="s">
-        <v>183</v>
       </c>
       <c r="N2" s="9"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="21" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B3" s="17" t="s">
         <v>40</v>
@@ -2429,19 +2430,19 @@
         <v>42</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J3" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K3" s="17" t="s">
         <v>43</v>
       </c>
       <c r="L3" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M3" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="N3" s="9"/>
     </row>
@@ -2450,334 +2451,334 @@
         <v>26</v>
       </c>
       <c r="B4" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="D4" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="E4" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="F4" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="E4" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="F4" s="17" t="s">
+      <c r="G4" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="I4" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="J4" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="H4" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="I4" s="17" t="s">
+      <c r="K4" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="L4" s="17" t="s">
         <v>190</v>
       </c>
-      <c r="J4" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="K4" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="L4" s="17" t="s">
-        <v>191</v>
-      </c>
       <c r="M4" s="17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="N4" s="9"/>
     </row>
     <row r="5" spans="1:14" ht="33" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B5" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="K5" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="L5" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="M5" s="17" t="s">
         <v>296</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>296</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>296</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>296</v>
-      </c>
-      <c r="H5" s="17" t="s">
-        <v>296</v>
-      </c>
-      <c r="I5" s="17" t="s">
-        <v>296</v>
-      </c>
-      <c r="J5" s="17" t="s">
-        <v>296</v>
-      </c>
-      <c r="K5" s="17" t="s">
-        <v>297</v>
-      </c>
-      <c r="L5" s="17" t="s">
-        <v>297</v>
-      </c>
-      <c r="M5" s="17" t="s">
-        <v>297</v>
       </c>
       <c r="N5" s="9"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="B6" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="D6" s="17" t="s">
+      <c r="E6" s="17" t="s">
         <v>194</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="F6" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="G6" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="I6" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="G6" s="17" t="s">
+      <c r="J6" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="H6" s="17" t="s">
-        <v>196</v>
-      </c>
-      <c r="I6" s="17" t="s">
+      <c r="K6" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="L6" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="J6" s="17" t="s">
+      <c r="M6" s="17" t="s">
         <v>197</v>
-      </c>
-      <c r="K6" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="L6" s="17" t="s">
-        <v>198</v>
-      </c>
-      <c r="M6" s="17" t="s">
-        <v>198</v>
       </c>
       <c r="N6" s="9"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
+        <v>198</v>
+      </c>
+      <c r="B7" s="17" t="s">
         <v>199</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="C7" s="17" t="s">
+        <v>199</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="E7" s="17" t="s">
         <v>200</v>
       </c>
-      <c r="C7" s="17" t="s">
-        <v>200</v>
-      </c>
-      <c r="D7" s="17" t="s">
+      <c r="F7" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="I7" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="E7" s="17" t="s">
-        <v>201</v>
-      </c>
-      <c r="F7" s="17" t="s">
-        <v>202</v>
-      </c>
-      <c r="G7" s="17" t="s">
-        <v>202</v>
-      </c>
-      <c r="H7" s="17" t="s">
-        <v>202</v>
-      </c>
-      <c r="I7" s="17" t="s">
-        <v>196</v>
-      </c>
       <c r="J7" s="17" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="K7" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="L7" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M7" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N7" s="9"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="21" t="s">
+        <v>202</v>
+      </c>
+      <c r="B8" s="17" t="s">
         <v>203</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="C8" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="D8" s="17" t="s">
         <v>204</v>
       </c>
-      <c r="C8" s="17" t="s">
-        <v>204</v>
-      </c>
-      <c r="D8" s="17" t="s">
+      <c r="E8" s="17" t="s">
         <v>205</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="F8" s="17" t="s">
         <v>206</v>
       </c>
-      <c r="F8" s="17" t="s">
-        <v>207</v>
-      </c>
       <c r="G8" s="17" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I8" s="17" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="J8" s="17" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="L8" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="M8" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="N8" s="9"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="21" t="s">
+        <v>207</v>
+      </c>
+      <c r="B9" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="C9" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="I9" s="17" t="s">
         <v>209</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="J9" s="17" t="s">
         <v>209</v>
       </c>
-      <c r="D9" s="17" t="s">
-        <v>96</v>
-      </c>
-      <c r="E9" s="17" t="s">
-        <v>96</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="G9" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="H9" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="I9" s="17" t="s">
-        <v>210</v>
-      </c>
-      <c r="J9" s="17" t="s">
-        <v>210</v>
-      </c>
       <c r="K9" s="17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L9" s="17" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M9" s="17" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N9" s="9"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="21" t="s">
+        <v>210</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D10" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="B10" s="17" t="s">
-        <v>209</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>209</v>
-      </c>
-      <c r="D10" s="17" t="s">
-        <v>212</v>
-      </c>
       <c r="E10" s="17" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I10" s="17" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J10" s="17" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K10" s="17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L10" s="17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="M10" s="17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="N10" s="9"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
+        <v>212</v>
+      </c>
+      <c r="B11" s="17" t="s">
         <v>213</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="C11" s="17" t="s">
+        <v>213</v>
+      </c>
+      <c r="D11" s="17" t="s">
         <v>214</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="E11" s="17" t="s">
         <v>214</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="F11" s="17" t="s">
         <v>215</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="G11" s="17" t="s">
         <v>215</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="H11" s="17" t="s">
+        <v>215</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="J11" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K11" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="L11" s="17" t="s">
         <v>216</v>
       </c>
-      <c r="G11" s="17" t="s">
+      <c r="M11" s="17" t="s">
         <v>216</v>
-      </c>
-      <c r="H11" s="17" t="s">
-        <v>216</v>
-      </c>
-      <c r="I11" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="J11" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="K11" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="L11" s="17" t="s">
-        <v>217</v>
-      </c>
-      <c r="M11" s="17" t="s">
-        <v>217</v>
       </c>
       <c r="N11" s="9"/>
     </row>
@@ -2786,40 +2787,40 @@
         <v>58</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I12" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="J12" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="K12" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="L12" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="M12" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="N12" s="9"/>
     </row>
@@ -2828,82 +2829,82 @@
         <v>59</v>
       </c>
       <c r="B13" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="D13" s="17" t="s">
         <v>219</v>
       </c>
-      <c r="C13" s="17" t="s">
-        <v>219</v>
-      </c>
-      <c r="D13" s="17" t="s">
+      <c r="E13" s="17" t="s">
         <v>220</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="F13" s="17" t="s">
         <v>221</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="G13" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="H13" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="I13" s="17" t="s">
         <v>222</v>
       </c>
-      <c r="G13" s="17" t="s">
+      <c r="J13" s="17" t="s">
         <v>222</v>
       </c>
-      <c r="H13" s="17" t="s">
-        <v>222</v>
-      </c>
-      <c r="I13" s="17" t="s">
+      <c r="K13" s="17" t="s">
         <v>223</v>
       </c>
-      <c r="J13" s="17" t="s">
-        <v>223</v>
-      </c>
-      <c r="K13" s="17" t="s">
+      <c r="L13" s="17" t="s">
         <v>224</v>
       </c>
-      <c r="L13" s="17" t="s">
-        <v>225</v>
-      </c>
       <c r="M13" s="17" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="N13" s="9"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="21" t="s">
+        <v>225</v>
+      </c>
+      <c r="B14" s="17" t="s">
         <v>226</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="C14" s="17" t="s">
         <v>227</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="D14" s="17" t="s">
         <v>228</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="E14" s="17" t="s">
+        <v>228</v>
+      </c>
+      <c r="F14" s="17" t="s">
         <v>229</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="G14" s="17" t="s">
         <v>229</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="H14" s="17" t="s">
+        <v>229</v>
+      </c>
+      <c r="I14" s="17" t="s">
         <v>230</v>
       </c>
-      <c r="G14" s="17" t="s">
+      <c r="J14" s="17" t="s">
         <v>230</v>
       </c>
-      <c r="H14" s="17" t="s">
-        <v>230</v>
-      </c>
-      <c r="I14" s="17" t="s">
+      <c r="K14" s="17" t="s">
         <v>231</v>
       </c>
-      <c r="J14" s="17" t="s">
-        <v>231</v>
-      </c>
-      <c r="K14" s="17" t="s">
+      <c r="L14" s="17" t="s">
         <v>232</v>
       </c>
-      <c r="L14" s="17" t="s">
-        <v>233</v>
-      </c>
       <c r="M14" s="17" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="N14" s="9"/>
     </row>
@@ -2912,88 +2913,88 @@
         <v>60</v>
       </c>
       <c r="B15" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="G15" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="I15" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="J15" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="K15" s="17" t="s">
         <v>234</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="L15" s="17" t="s">
         <v>234</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="M15" s="17" t="s">
         <v>234</v>
-      </c>
-      <c r="E15" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="F15" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="G15" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="H15" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="I15" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="J15" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="K15" s="17" t="s">
-        <v>235</v>
-      </c>
-      <c r="L15" s="17" t="s">
-        <v>235</v>
-      </c>
-      <c r="M15" s="17" t="s">
-        <v>235</v>
       </c>
       <c r="N15" s="9"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
+        <v>235</v>
+      </c>
+      <c r="B16" s="17" t="s">
         <v>236</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="C16" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="F16" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="G16" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="H16" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="E16" s="17" t="s">
-        <v>237</v>
-      </c>
-      <c r="F16" s="17" t="s">
+      <c r="I16" s="17" t="s">
         <v>238</v>
       </c>
-      <c r="G16" s="17" t="s">
+      <c r="J16" s="17" t="s">
         <v>238</v>
       </c>
-      <c r="H16" s="17" t="s">
+      <c r="K16" s="17" t="s">
         <v>238</v>
       </c>
-      <c r="I16" s="17" t="s">
-        <v>239</v>
-      </c>
-      <c r="J16" s="17" t="s">
-        <v>239</v>
-      </c>
-      <c r="K16" s="17" t="s">
-        <v>239</v>
-      </c>
       <c r="L16" s="17" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="M16" s="17" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="N16" s="9"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="21" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B17" s="17" t="s">
         <v>54</v>
@@ -3035,337 +3036,337 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="B18" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="C18" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="D18" s="17" t="s">
         <v>242</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="E18" s="17" t="s">
         <v>242</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="F18" s="17" t="s">
         <v>243</v>
       </c>
-      <c r="E18" s="17" t="s">
-        <v>243</v>
-      </c>
-      <c r="F18" s="17" t="s">
+      <c r="G18" s="17" t="s">
         <v>244</v>
       </c>
-      <c r="G18" s="17" t="s">
+      <c r="H18" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="I18" s="17" t="s">
         <v>245</v>
       </c>
-      <c r="H18" s="17" t="s">
-        <v>245</v>
-      </c>
-      <c r="I18" s="17" t="s">
+      <c r="J18" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="K18" s="17" t="s">
         <v>246</v>
       </c>
-      <c r="J18" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="K18" s="17" t="s">
+      <c r="L18" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="M18" s="17" t="s">
         <v>247</v>
-      </c>
-      <c r="L18" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="M18" s="17" t="s">
-        <v>248</v>
       </c>
       <c r="N18" s="9"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="21" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B19" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="D19" s="17" t="s">
         <v>242</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="E19" s="17" t="s">
         <v>242</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="F19" s="17" t="s">
         <v>243</v>
       </c>
-      <c r="E19" s="17" t="s">
-        <v>243</v>
-      </c>
-      <c r="F19" s="17" t="s">
+      <c r="G19" s="17" t="s">
         <v>244</v>
       </c>
-      <c r="G19" s="17" t="s">
+      <c r="H19" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="I19" s="17" t="s">
         <v>245</v>
       </c>
-      <c r="H19" s="17" t="s">
-        <v>245</v>
-      </c>
-      <c r="I19" s="17" t="s">
+      <c r="J19" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="K19" s="17" t="s">
         <v>246</v>
       </c>
-      <c r="J19" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="K19" s="17" t="s">
+      <c r="L19" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="M19" s="17" t="s">
         <v>247</v>
-      </c>
-      <c r="L19" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="M19" s="17" t="s">
-        <v>248</v>
       </c>
       <c r="N19" s="9"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="B20" s="17" t="s">
         <v>250</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="C20" s="17" t="s">
+        <v>250</v>
+      </c>
+      <c r="D20" s="17" t="s">
         <v>251</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="E20" s="17" t="s">
         <v>251</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="F20" s="17" t="s">
         <v>252</v>
       </c>
-      <c r="E20" s="17" t="s">
-        <v>252</v>
-      </c>
-      <c r="F20" s="17" t="s">
+      <c r="G20" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="G20" s="17" t="s">
+      <c r="H20" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="I20" s="17" t="s">
         <v>254</v>
       </c>
-      <c r="H20" s="17" t="s">
+      <c r="J20" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="K20" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="L20" s="17" t="s">
         <v>254</v>
       </c>
-      <c r="I20" s="17" t="s">
+      <c r="M20" s="17" t="s">
         <v>255</v>
-      </c>
-      <c r="J20" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="K20" s="17" t="s">
-        <v>254</v>
-      </c>
-      <c r="L20" s="17" t="s">
-        <v>255</v>
-      </c>
-      <c r="M20" s="17" t="s">
-        <v>256</v>
       </c>
       <c r="N20" s="9"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="21" t="s">
+        <v>256</v>
+      </c>
+      <c r="B21" s="17" t="s">
         <v>257</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="C21" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="D21" s="17" t="s">
         <v>258</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="E21" s="17" t="s">
         <v>258</v>
       </c>
-      <c r="D21" s="17" t="s">
+      <c r="F21" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="H21" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="I21" s="17" t="s">
         <v>259</v>
       </c>
-      <c r="E21" s="17" t="s">
-        <v>259</v>
-      </c>
-      <c r="F21" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="G21" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="H21" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="I21" s="17" t="s">
+      <c r="J21" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="K21" s="17" t="s">
         <v>260</v>
       </c>
-      <c r="J21" s="17" t="s">
-        <v>116</v>
-      </c>
-      <c r="K21" s="17" t="s">
+      <c r="L21" s="17" t="s">
         <v>261</v>
       </c>
-      <c r="L21" s="17" t="s">
+      <c r="M21" s="17" t="s">
         <v>262</v>
-      </c>
-      <c r="M21" s="17" t="s">
-        <v>263</v>
       </c>
       <c r="N21" s="9"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="21" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B22" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="D22" s="17" t="s">
         <v>258</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="E22" s="17" t="s">
         <v>258</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="F22" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="G22" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="H22" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="I22" s="17" t="s">
         <v>259</v>
       </c>
-      <c r="E22" s="17" t="s">
-        <v>259</v>
-      </c>
-      <c r="F22" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="G22" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="H22" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="I22" s="17" t="s">
+      <c r="J22" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="K22" s="17" t="s">
         <v>260</v>
       </c>
-      <c r="J22" s="17" t="s">
-        <v>116</v>
-      </c>
-      <c r="K22" s="17" t="s">
+      <c r="L22" s="17" t="s">
         <v>261</v>
       </c>
-      <c r="L22" s="17" t="s">
+      <c r="M22" s="17" t="s">
         <v>262</v>
-      </c>
-      <c r="M22" s="17" t="s">
-        <v>263</v>
       </c>
       <c r="N22" s="9"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="21" t="s">
+        <v>264</v>
+      </c>
+      <c r="B23" s="17" t="s">
         <v>265</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="C23" s="17" t="s">
+        <v>265</v>
+      </c>
+      <c r="D23" s="17" t="s">
         <v>266</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="E23" s="17" t="s">
         <v>266</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="F23" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="H23" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="I23" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="J23" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="K23" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="L23" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="M23" s="17" t="s">
         <v>267</v>
-      </c>
-      <c r="E23" s="17" t="s">
-        <v>267</v>
-      </c>
-      <c r="F23" s="17" t="s">
-        <v>258</v>
-      </c>
-      <c r="G23" s="17" t="s">
-        <v>258</v>
-      </c>
-      <c r="H23" s="17" t="s">
-        <v>258</v>
-      </c>
-      <c r="I23" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="J23" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="K23" s="17" t="s">
-        <v>258</v>
-      </c>
-      <c r="L23" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="M23" s="17" t="s">
-        <v>268</v>
       </c>
       <c r="N23" s="9"/>
     </row>
     <row r="24" spans="1:14" ht="33" x14ac:dyDescent="0.3">
       <c r="A24" s="21" t="s">
+        <v>268</v>
+      </c>
+      <c r="B24" s="17" t="s">
         <v>269</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="C24" s="17" t="s">
+        <v>292</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>293</v>
+      </c>
+      <c r="E24" s="17" t="s">
+        <v>293</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="G24" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="H24" s="17" t="s">
+        <v>293</v>
+      </c>
+      <c r="I24" s="17" t="s">
+        <v>297</v>
+      </c>
+      <c r="J24" s="17" t="s">
+        <v>297</v>
+      </c>
+      <c r="K24" s="17" t="s">
         <v>270</v>
       </c>
-      <c r="C24" s="17" t="s">
-        <v>293</v>
-      </c>
-      <c r="D24" s="17" t="s">
-        <v>294</v>
-      </c>
-      <c r="E24" s="17" t="s">
-        <v>294</v>
-      </c>
-      <c r="F24" s="17" t="s">
+      <c r="L24" s="17" t="s">
         <v>270</v>
       </c>
-      <c r="G24" s="17" t="s">
+      <c r="M24" s="17" t="s">
         <v>270</v>
-      </c>
-      <c r="H24" s="17" t="s">
-        <v>294</v>
-      </c>
-      <c r="I24" s="17" t="s">
-        <v>298</v>
-      </c>
-      <c r="J24" s="17" t="s">
-        <v>298</v>
-      </c>
-      <c r="K24" s="17" t="s">
-        <v>271</v>
-      </c>
-      <c r="L24" s="17" t="s">
-        <v>271</v>
-      </c>
-      <c r="M24" s="17" t="s">
-        <v>271</v>
       </c>
       <c r="N24" s="9"/>
     </row>
     <row r="25" spans="1:14" ht="33" x14ac:dyDescent="0.3">
       <c r="A25" s="21" t="s">
+        <v>271</v>
+      </c>
+      <c r="B25" s="17" t="s">
         <v>272</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="C25" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="H25" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="I25" s="22" t="s">
+        <v>298</v>
+      </c>
+      <c r="J25" s="22" t="s">
+        <v>298</v>
+      </c>
+      <c r="K25" s="17" t="s">
         <v>273</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="L25" s="17" t="s">
         <v>273</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="M25" s="17" t="s">
         <v>273</v>
-      </c>
-      <c r="E25" s="17" t="s">
-        <v>273</v>
-      </c>
-      <c r="F25" s="17" t="s">
-        <v>273</v>
-      </c>
-      <c r="G25" s="17" t="s">
-        <v>273</v>
-      </c>
-      <c r="H25" s="17" t="s">
-        <v>273</v>
-      </c>
-      <c r="I25" s="22" t="s">
-        <v>299</v>
-      </c>
-      <c r="J25" s="22" t="s">
-        <v>299</v>
-      </c>
-      <c r="K25" s="17" t="s">
-        <v>274</v>
-      </c>
-      <c r="L25" s="17" t="s">
-        <v>274</v>
-      </c>
-      <c r="M25" s="17" t="s">
-        <v>274</v>
       </c>
       <c r="N25" s="9"/>
     </row>
@@ -3413,43 +3414,43 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="21" t="s">
+        <v>274</v>
+      </c>
+      <c r="B27" s="17" t="s">
         <v>275</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="C27" s="17" t="s">
         <v>276</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="D27" s="17" t="s">
         <v>277</v>
       </c>
-      <c r="D27" s="17" t="s">
+      <c r="E27" s="17" t="s">
         <v>278</v>
       </c>
-      <c r="E27" s="17" t="s">
+      <c r="F27" s="17" t="s">
         <v>279</v>
       </c>
-      <c r="F27" s="17" t="s">
+      <c r="G27" s="17" t="s">
         <v>280</v>
       </c>
-      <c r="G27" s="17" t="s">
+      <c r="H27" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="I27" s="17" t="s">
         <v>281</v>
       </c>
-      <c r="H27" s="17" t="s">
-        <v>248</v>
-      </c>
-      <c r="I27" s="17" t="s">
+      <c r="J27" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="K27" s="17" t="s">
         <v>282</v>
       </c>
-      <c r="J27" s="17" t="s">
-        <v>146</v>
-      </c>
-      <c r="K27" s="17" t="s">
+      <c r="L27" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="M27" s="17" t="s">
         <v>283</v>
-      </c>
-      <c r="L27" s="17" t="s">
-        <v>197</v>
-      </c>
-      <c r="M27" s="17" t="s">
-        <v>284</v>
       </c>
       <c r="N27" s="9"/>
     </row>
@@ -3458,82 +3459,82 @@
         <v>32</v>
       </c>
       <c r="B28" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="E28" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="F28" s="17" t="s">
         <v>285</v>
       </c>
-      <c r="C28" s="17" t="s">
+      <c r="G28" s="17" t="s">
         <v>285</v>
       </c>
-      <c r="D28" s="17" t="s">
+      <c r="H28" s="17" t="s">
         <v>285</v>
       </c>
-      <c r="E28" s="17" t="s">
+      <c r="I28" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="J28" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="K28" s="17" t="s">
+        <v>287</v>
+      </c>
+      <c r="L28" s="17" t="s">
         <v>285</v>
       </c>
-      <c r="F28" s="17" t="s">
-        <v>286</v>
-      </c>
-      <c r="G28" s="17" t="s">
-        <v>286</v>
-      </c>
-      <c r="H28" s="17" t="s">
-        <v>286</v>
-      </c>
-      <c r="I28" s="17" t="s">
+      <c r="M28" s="17" t="s">
         <v>287</v>
-      </c>
-      <c r="J28" s="17" t="s">
-        <v>287</v>
-      </c>
-      <c r="K28" s="17" t="s">
-        <v>288</v>
-      </c>
-      <c r="L28" s="17" t="s">
-        <v>286</v>
-      </c>
-      <c r="M28" s="17" t="s">
-        <v>288</v>
       </c>
       <c r="N28" s="9"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="21" t="s">
+        <v>288</v>
+      </c>
+      <c r="B29" s="17" t="s">
         <v>289</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="C29" s="17" t="s">
+        <v>289</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>289</v>
+      </c>
+      <c r="E29" s="17" t="s">
+        <v>289</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>289</v>
+      </c>
+      <c r="G29" s="17" t="s">
+        <v>289</v>
+      </c>
+      <c r="H29" s="17" t="s">
+        <v>289</v>
+      </c>
+      <c r="I29" s="17" t="s">
+        <v>289</v>
+      </c>
+      <c r="J29" s="17" t="s">
+        <v>289</v>
+      </c>
+      <c r="K29" s="17" t="s">
         <v>290</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="L29" s="17" t="s">
         <v>290</v>
       </c>
-      <c r="D29" s="17" t="s">
+      <c r="M29" s="17" t="s">
         <v>290</v>
-      </c>
-      <c r="E29" s="17" t="s">
-        <v>290</v>
-      </c>
-      <c r="F29" s="17" t="s">
-        <v>290</v>
-      </c>
-      <c r="G29" s="17" t="s">
-        <v>290</v>
-      </c>
-      <c r="H29" s="17" t="s">
-        <v>290</v>
-      </c>
-      <c r="I29" s="17" t="s">
-        <v>290</v>
-      </c>
-      <c r="J29" s="17" t="s">
-        <v>290</v>
-      </c>
-      <c r="K29" s="17" t="s">
-        <v>291</v>
-      </c>
-      <c r="L29" s="17" t="s">
-        <v>291</v>
-      </c>
-      <c r="M29" s="17" t="s">
-        <v>291</v>
       </c>
       <c r="N29" s="9"/>
     </row>
@@ -3542,40 +3543,40 @@
         <v>37</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F30" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G30" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H30" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="I30" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J30" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K30" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="L30" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="M30" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="N30" s="9"/>
     </row>
@@ -5015,58 +5016,58 @@
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26" s="21" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="H26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="I26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="J26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="K26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="M26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="N26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="O26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="Q26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="R26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
   </sheetData>
@@ -5117,25 +5118,25 @@
         <v>18</v>
       </c>
       <c r="B2" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="F2" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="H2" s="12" t="s">
         <v>88</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="H2" s="12" t="s">
-        <v>89</v>
       </c>
       <c r="I2" s="9"/>
     </row>
@@ -5144,25 +5145,25 @@
         <v>19</v>
       </c>
       <c r="B3" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="E3" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="G3" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="H3" s="13" t="s">
         <v>93</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="G3" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="H3" s="13" t="s">
-        <v>94</v>
       </c>
       <c r="I3" s="9"/>
     </row>
@@ -5171,25 +5172,25 @@
         <v>20</v>
       </c>
       <c r="B4" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="D4" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="F4" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="G4" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>99</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>100</v>
       </c>
       <c r="I4" s="9"/>
     </row>
@@ -5198,25 +5199,25 @@
         <v>21</v>
       </c>
       <c r="B5" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="C5" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="D5" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="E5" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="F5" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="G5" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="H5" s="13" t="s">
         <v>107</v>
-      </c>
-      <c r="H5" s="13" t="s">
-        <v>108</v>
       </c>
       <c r="I5" s="9"/>
     </row>
@@ -5225,25 +5226,25 @@
         <v>22</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I6" s="9"/>
     </row>
@@ -5252,25 +5253,25 @@
         <v>56</v>
       </c>
       <c r="B7" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="D7" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="F7" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="G7" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="H7" s="13" t="s">
         <v>113</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>114</v>
       </c>
       <c r="I7" s="9"/>
     </row>
@@ -5360,25 +5361,25 @@
         <v>25</v>
       </c>
       <c r="B11" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="C11" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="D11" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="F11" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="G11" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="H11" s="13" t="s">
         <v>117</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="H11" s="13" t="s">
-        <v>118</v>
       </c>
       <c r="I11" s="9"/>
     </row>
@@ -5387,25 +5388,25 @@
         <v>26</v>
       </c>
       <c r="B12" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>122</v>
-      </c>
       <c r="D12" s="12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I12" s="9"/>
     </row>
@@ -5414,25 +5415,25 @@
         <v>61</v>
       </c>
       <c r="B13" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="C13" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="D13" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="F13" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="G13" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="H13" s="13" t="s">
         <v>126</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="H13" s="13" t="s">
-        <v>127</v>
       </c>
       <c r="I13" s="9"/>
     </row>
@@ -5441,25 +5442,25 @@
         <v>62</v>
       </c>
       <c r="B14" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="C14" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="D14" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F14" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="G14" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="H14" s="12" t="s">
         <v>131</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="G14" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="H14" s="12" t="s">
-        <v>132</v>
       </c>
       <c r="I14" s="9"/>
     </row>
@@ -5495,25 +5496,25 @@
         <v>28</v>
       </c>
       <c r="B16" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="D16" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="E16" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="F16" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="F16" s="13" t="s">
+      <c r="G16" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="G16" s="13" t="s">
-        <v>139</v>
-      </c>
       <c r="H16" s="13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I16" s="9"/>
     </row>
@@ -5522,25 +5523,25 @@
         <v>29</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I17" s="9"/>
     </row>
@@ -5549,25 +5550,25 @@
         <v>66</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I18" s="9"/>
     </row>
@@ -5630,25 +5631,25 @@
         <v>30</v>
       </c>
       <c r="B21" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="C21" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="C21" s="12" t="s">
-        <v>149</v>
-      </c>
       <c r="D21" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I21" s="9"/>
     </row>
@@ -5684,25 +5685,25 @@
         <v>31</v>
       </c>
       <c r="B23" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C23" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="D23" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="E23" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="F23" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="G23" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="F23" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="G23" s="12" t="s">
+      <c r="H23" s="12" t="s">
         <v>154</v>
-      </c>
-      <c r="H23" s="12" t="s">
-        <v>155</v>
       </c>
       <c r="I23" s="9"/>
     </row>
@@ -5762,28 +5763,28 @@
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26" s="21" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="H26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="I26" s="17"/>
       <c r="J26" s="17"/>
@@ -5822,25 +5823,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>305</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>306</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>79</v>
@@ -5852,13 +5853,13 @@
         <v>81</v>
       </c>
       <c r="L1" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -5866,43 +5867,43 @@
         <v>18</v>
       </c>
       <c r="B2" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="23" t="s">
+      <c r="D2" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="D2" s="23" t="s">
+      <c r="E2" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="E2" s="23" t="s">
+      <c r="F2" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="G2" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="H2" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="F2" s="23" t="s">
-        <v>87</v>
-      </c>
-      <c r="G2" s="23" t="s">
+      <c r="I2" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="H2" s="23" t="s">
+      <c r="J2" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="I2" s="23" t="s">
+      <c r="K2" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="L2" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="M2" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="23" t="s">
+      <c r="N2" s="23" t="s">
         <v>90</v>
-      </c>
-      <c r="K2" s="23" t="s">
-        <v>91</v>
-      </c>
-      <c r="L2" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="M2" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="N2" s="23" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -5910,43 +5911,43 @@
         <v>19</v>
       </c>
       <c r="B3" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="E3" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="G3" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="H3" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="E3" s="23" t="s">
+      <c r="I3" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="F3" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="G3" s="23" t="s">
-        <v>93</v>
-      </c>
-      <c r="H3" s="23" t="s">
+      <c r="J3" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="K3" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="L3" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="I3" s="23" t="s">
+      <c r="M3" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="J3" s="23" t="s">
+      <c r="N3" s="23" t="s">
         <v>96</v>
-      </c>
-      <c r="K3" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="L3" s="23" t="s">
-        <v>95</v>
-      </c>
-      <c r="M3" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="N3" s="23" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -5954,175 +5955,175 @@
         <v>20</v>
       </c>
       <c r="B4" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="F4" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="G4" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="H4" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="I4" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="G4" s="23" t="s">
+      <c r="J4" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="K4" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="I4" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="J4" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="K4" s="23" t="s">
-        <v>101</v>
-      </c>
       <c r="L4" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M4" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="N4" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="B5" s="23" t="s">
         <v>307</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="C5" s="23" t="s">
         <v>308</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="D5" s="23" t="s">
         <v>309</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="E5" s="23" t="s">
         <v>310</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="F5" s="23" t="s">
         <v>311</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="G5" s="23" t="s">
         <v>312</v>
       </c>
-      <c r="G5" s="23" t="s">
+      <c r="H5" s="23" t="s">
         <v>313</v>
       </c>
-      <c r="H5" s="23" t="s">
-        <v>314</v>
-      </c>
       <c r="I5" s="23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K5" s="23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L5" s="23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M5" s="23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N5" s="23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="B6" s="23" t="s">
         <v>315</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="C6" s="23" t="s">
         <v>316</v>
       </c>
-      <c r="C6" s="23" t="s">
-        <v>317</v>
-      </c>
       <c r="D6" s="23" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K6" s="23" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="L6" s="23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M6" s="23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N6" s="23" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B7" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="D7" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="F7" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="G7" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="H7" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="I7" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="J7" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="H7" s="23" t="s">
+      <c r="K7" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="I7" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="J7" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="K7" s="23" t="s">
-        <v>115</v>
-      </c>
       <c r="L7" s="23" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M7" s="23" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="N7" s="23" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -6259,90 +6260,90 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B11" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="F11" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="C11" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="F11" s="23" t="s">
+      <c r="G11" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="I11" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="G11" s="23" t="s">
+      <c r="J11" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="H11" s="23" t="s">
+      <c r="K11" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="I11" s="23" t="s">
+      <c r="L11" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="J11" s="23" t="s">
+      <c r="M11" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="K11" s="23" t="s">
+      <c r="N11" s="23" t="s">
         <v>119</v>
-      </c>
-      <c r="L11" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="M11" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="N11" s="23" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B12" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="C12" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="C12" s="23" t="s">
-        <v>188</v>
-      </c>
       <c r="D12" s="23" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I12" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="J12" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="K12" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="L12" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="J12" s="23" t="s">
+      <c r="M12" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="K12" s="23" t="s">
+      <c r="N12" s="23" t="s">
         <v>123</v>
-      </c>
-      <c r="L12" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="M12" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="N12" s="23" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
@@ -6350,43 +6351,43 @@
         <v>61</v>
       </c>
       <c r="B13" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="C13" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="D13" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F13" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="G13" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="E13" s="23" t="s">
+      <c r="H13" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="F13" s="23" t="s">
+      <c r="I13" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="J13" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="H13" s="23" t="s">
+      <c r="K13" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="I13" s="23" t="s">
+      <c r="L13" s="23" t="s">
         <v>128</v>
       </c>
-      <c r="J13" s="23" t="s">
+      <c r="M13" s="23" t="s">
         <v>128</v>
       </c>
-      <c r="K13" s="23" t="s">
+      <c r="N13" s="23" t="s">
         <v>128</v>
-      </c>
-      <c r="L13" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="M13" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="N13" s="23" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -6394,43 +6395,43 @@
         <v>62</v>
       </c>
       <c r="B14" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="C14" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="D14" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="F14" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="G14" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="E14" s="23" t="s">
+      <c r="H14" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="F14" s="23" t="s">
+      <c r="I14" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="G14" s="23" t="s">
+      <c r="J14" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="H14" s="23" t="s">
+      <c r="K14" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="I14" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="K14" s="23" t="s">
-        <v>133</v>
-      </c>
       <c r="L14" s="23" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="M14" s="23" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N14" s="23" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="33" x14ac:dyDescent="0.3">
@@ -6438,25 +6439,25 @@
         <v>27</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="I15" s="7" t="s">
         <v>71</v>
@@ -6482,43 +6483,43 @@
         <v>28</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D16" s="23" t="s">
+        <v>320</v>
+      </c>
+      <c r="E16" s="23" t="s">
         <v>321</v>
       </c>
-      <c r="E16" s="23" t="s">
+      <c r="F16" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>321</v>
+      </c>
+      <c r="H16" s="23" t="s">
         <v>322</v>
       </c>
-      <c r="F16" s="23" t="s">
+      <c r="I16" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="G16" s="23" t="s">
-        <v>322</v>
-      </c>
-      <c r="H16" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="I16" s="23" t="s">
+      <c r="J16" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="J16" s="23" t="s">
+      <c r="K16" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="K16" s="23" t="s">
+      <c r="L16" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="L16" s="23" t="s">
+      <c r="M16" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="M16" s="23" t="s">
+      <c r="N16" s="23" t="s">
         <v>144</v>
-      </c>
-      <c r="N16" s="23" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="33" x14ac:dyDescent="0.3">
@@ -6702,43 +6703,43 @@
         <v>30</v>
       </c>
       <c r="B21" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="C21" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="D21" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="E21" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="G21" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="H21" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="I21" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="D21" s="23" t="s">
+      <c r="J21" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="E21" s="23" t="s">
+      <c r="K21" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="F21" s="23" t="s">
-        <v>149</v>
-      </c>
-      <c r="G21" s="23" t="s">
-        <v>149</v>
-      </c>
-      <c r="H21" s="23" t="s">
-        <v>149</v>
-      </c>
-      <c r="I21" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="J21" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="K21" s="23" t="s">
-        <v>150</v>
-      </c>
       <c r="L21" s="23" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M21" s="23" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="N21" s="23" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
@@ -6790,43 +6791,43 @@
         <v>31</v>
       </c>
       <c r="B23" s="23" t="s">
+        <v>323</v>
+      </c>
+      <c r="C23" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="D23" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="E23" s="23" t="s">
+        <v>325</v>
+      </c>
+      <c r="F23" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="G23" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="H23" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="I23" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="J23" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="K23" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="L23" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="D23" s="23" t="s">
-        <v>325</v>
-      </c>
-      <c r="E23" s="23" t="s">
-        <v>326</v>
-      </c>
-      <c r="F23" s="23" t="s">
+      <c r="M23" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="N23" s="23" t="s">
         <v>152</v>
-      </c>
-      <c r="G23" s="23" t="s">
-        <v>327</v>
-      </c>
-      <c r="H23" s="23" t="s">
-        <v>154</v>
-      </c>
-      <c r="I23" s="23" t="s">
-        <v>156</v>
-      </c>
-      <c r="J23" s="23" t="s">
-        <v>157</v>
-      </c>
-      <c r="K23" s="23" t="s">
-        <v>151</v>
-      </c>
-      <c r="L23" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="M23" s="23" t="s">
-        <v>156</v>
-      </c>
-      <c r="N23" s="23" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
@@ -6919,46 +6920,46 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="21" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="H26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="I26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="J26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="K26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="M26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="N26" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>